<commit_message>
Restructure session 5 by chart family with build steps, and tidy team projects
Session 5 groups similar charts on interactive slides (bar/column variants,
pie/donut, waterfall/funnel, combo, card/gauge), follows each explanation
with a "Construiește în Power BI" slide listing the exact fields per well,
and adds a design and storytelling part. Team project briefs are simplified,
their sheet names no longer reveal fact vs dimension, and product weights
and two fractional quantities are corrected. The old shared dirty files and
the 4-page report are removed from the published folder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Curs Oficial/sesiuni/s05/echipa_albastru/Clienti.xlsx
+++ b/Curs Oficial/sesiuni/s05/echipa_albastru/Clienti.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dim_Clienti" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clienti" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -422,15 +422,6 @@
           <t>Baza clienti DMS</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -438,15 +429,6 @@
           <t>backup martie 2025</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1914,15 +1896,6 @@
           <t>— export terminat —</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>